<commit_message>
Windows: Minor update to v1.7 before second release
</commit_message>
<xml_diff>
--- a/Data-Examples/Ag2S/Ag2S_Kfitting.xlsx
+++ b/Data-Examples/Ag2S/Ag2S_Kfitting.xlsx
@@ -262,7 +262,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7210425" cy="4067175"/>
+    <ext cx="5667375" cy="3238500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -899,9 +899,99 @@
       <c r="G2" t="n">
         <v>708507</v>
       </c>
-      <c r="X2" s="4" t="inlineStr">
-        <is>
-          <t>Please cite KherveFitting software: Kerherve G. et al. Surface and Interface Analysis (2025) TBD</t>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Y2" s="6" t="inlineStr">
+        <is>
+          <t>Cu2p .</t>
+        </is>
+      </c>
+      <c r="Z2" s="6" t="inlineStr">
+        <is>
+          <t>932.86</t>
+        </is>
+      </c>
+      <c r="AA2" s="6" t="inlineStr">
+        <is>
+          <t>72055.19</t>
+        </is>
+      </c>
+      <c r="AB2" s="6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AC2" s="6" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="AD2" s="6" t="inlineStr">
+        <is>
+          <t>252036.38</t>
+        </is>
+      </c>
+      <c r="AE2" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AF2" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AG2" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AH2" s="6" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="AI2" s="6" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="AJ2" s="6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK2" s="6" t="inlineStr">
+        <is>
+          <t>Unfitted</t>
+        </is>
+      </c>
+      <c r="AL2" s="6" t="inlineStr">
+        <is>
+          <t>U2-Tougaard</t>
+        </is>
+      </c>
+      <c r="AM2" s="6" t="inlineStr">
+        <is>
+          <t>907.86</t>
+        </is>
+      </c>
+      <c r="AN2" s="6" t="inlineStr">
+        <is>
+          <t>957.86</t>
+        </is>
+      </c>
+      <c r="AO2" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AP2" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
@@ -928,6 +1018,57 @@
       <c r="G3" t="n">
         <v>705652</v>
       </c>
+      <c r="X3" s="7" t="inlineStr"/>
+      <c r="Y3" s="8" t="inlineStr"/>
+      <c r="Z3" s="8" t="inlineStr">
+        <is>
+          <t>-9.64:1350.36</t>
+        </is>
+      </c>
+      <c r="AA3" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AB3" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3.7</t>
+        </is>
+      </c>
+      <c r="AC3" s="8" t="inlineStr">
+        <is>
+          <t>5:80</t>
+        </is>
+      </c>
+      <c r="AD3" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AE3" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AF3" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AG3" s="8" t="inlineStr">
+        <is>
+          <t>0.01:2</t>
+        </is>
+      </c>
+      <c r="AH3" s="8" t="inlineStr"/>
+      <c r="AI3" s="8" t="inlineStr"/>
+      <c r="AJ3" s="8" t="inlineStr"/>
+      <c r="AK3" s="8" t="inlineStr"/>
+      <c r="AL3" s="8" t="inlineStr"/>
+      <c r="AM3" s="8" t="inlineStr"/>
+      <c r="AN3" s="8" t="inlineStr"/>
+      <c r="AO3" s="8" t="inlineStr"/>
+      <c r="AP3" s="8" t="inlineStr"/>
       <c r="AS3" t="inlineStr">
         <is>
           <t>Number of Scans</t>
@@ -952,6 +1093,101 @@
       <c r="G4" t="n">
         <v>698369</v>
       </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>Ag3d .</t>
+        </is>
+      </c>
+      <c r="Z4" s="6" t="inlineStr">
+        <is>
+          <t>368.36</t>
+        </is>
+      </c>
+      <c r="AA4" s="6" t="inlineStr">
+        <is>
+          <t>1210466.15</t>
+        </is>
+      </c>
+      <c r="AB4" s="6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AC4" s="6" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="AD4" s="6" t="inlineStr">
+        <is>
+          <t>4738252.91</t>
+        </is>
+      </c>
+      <c r="AE4" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AF4" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AG4" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AH4" s="6" t="inlineStr">
+        <is>
+          <t>45.3</t>
+        </is>
+      </c>
+      <c r="AI4" s="6" t="inlineStr">
+        <is>
+          <t>1879.99</t>
+        </is>
+      </c>
+      <c r="AJ4" s="6" t="inlineStr">
+        <is>
+          <t>-564.50</t>
+        </is>
+      </c>
+      <c r="AK4" s="6" t="inlineStr">
+        <is>
+          <t>Unfitted</t>
+        </is>
+      </c>
+      <c r="AL4" s="6" t="inlineStr">
+        <is>
+          <t>U2-Tougaard</t>
+        </is>
+      </c>
+      <c r="AM4" s="6" t="inlineStr">
+        <is>
+          <t>359.86</t>
+        </is>
+      </c>
+      <c r="AN4" s="6" t="inlineStr">
+        <is>
+          <t>385.36</t>
+        </is>
+      </c>
+      <c r="AO4" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AP4" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
       <c r="AS4" t="inlineStr">
         <is>
           <t>Source Gun Type</t>
@@ -976,6 +1212,57 @@
       <c r="G5" t="n">
         <v>704281</v>
       </c>
+      <c r="X5" s="7" t="inlineStr"/>
+      <c r="Y5" s="8" t="inlineStr"/>
+      <c r="Z5" s="8" t="inlineStr">
+        <is>
+          <t>-9.64:1350.36</t>
+        </is>
+      </c>
+      <c r="AA5" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AB5" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3.7</t>
+        </is>
+      </c>
+      <c r="AC5" s="8" t="inlineStr">
+        <is>
+          <t>5:80</t>
+        </is>
+      </c>
+      <c r="AD5" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AE5" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AF5" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AG5" s="8" t="inlineStr">
+        <is>
+          <t>0.01:2</t>
+        </is>
+      </c>
+      <c r="AH5" s="8" t="inlineStr"/>
+      <c r="AI5" s="8" t="inlineStr"/>
+      <c r="AJ5" s="8" t="inlineStr"/>
+      <c r="AK5" s="8" t="inlineStr"/>
+      <c r="AL5" s="8" t="inlineStr"/>
+      <c r="AM5" s="8" t="inlineStr"/>
+      <c r="AN5" s="8" t="inlineStr"/>
+      <c r="AO5" s="8" t="inlineStr"/>
+      <c r="AP5" s="8" t="inlineStr"/>
       <c r="AS5" t="inlineStr">
         <is>
           <t>Spot Size</t>
@@ -1000,6 +1287,101 @@
       <c r="G6" t="n">
         <v>688203</v>
       </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y6" s="6" t="inlineStr">
+        <is>
+          <t>C1s .</t>
+        </is>
+      </c>
+      <c r="Z6" s="6" t="inlineStr">
+        <is>
+          <t>284.86</t>
+        </is>
+      </c>
+      <c r="AA6" s="6" t="inlineStr">
+        <is>
+          <t>49486.54</t>
+        </is>
+      </c>
+      <c r="AB6" s="6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AC6" s="6" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="AD6" s="6" t="inlineStr">
+        <is>
+          <t>121979.93</t>
+        </is>
+      </c>
+      <c r="AE6" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AF6" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AG6" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AH6" s="6" t="inlineStr">
+        <is>
+          <t>27.4</t>
+        </is>
+      </c>
+      <c r="AI6" s="6" t="inlineStr">
+        <is>
+          <t>48.40</t>
+        </is>
+      </c>
+      <c r="AJ6" s="6" t="inlineStr">
+        <is>
+          <t>-648.00</t>
+        </is>
+      </c>
+      <c r="AK6" s="6" t="inlineStr">
+        <is>
+          <t>Unfitted</t>
+        </is>
+      </c>
+      <c r="AL6" s="6" t="inlineStr">
+        <is>
+          <t>U2-Tougaard</t>
+        </is>
+      </c>
+      <c r="AM6" s="6" t="inlineStr">
+        <is>
+          <t>273.36</t>
+        </is>
+      </c>
+      <c r="AN6" s="6" t="inlineStr">
+        <is>
+          <t>301.86</t>
+        </is>
+      </c>
+      <c r="AO6" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AP6" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
       <c r="AS6" t="inlineStr">
         <is>
           <t>Lens Mode</t>
@@ -1024,6 +1406,57 @@
       <c r="G7" t="n">
         <v>691612</v>
       </c>
+      <c r="X7" s="7" t="inlineStr"/>
+      <c r="Y7" s="8" t="inlineStr"/>
+      <c r="Z7" s="8" t="inlineStr">
+        <is>
+          <t>-9.64:1350.36</t>
+        </is>
+      </c>
+      <c r="AA7" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AB7" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3.7</t>
+        </is>
+      </c>
+      <c r="AC7" s="8" t="inlineStr">
+        <is>
+          <t>5:80</t>
+        </is>
+      </c>
+      <c r="AD7" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AE7" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AF7" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AG7" s="8" t="inlineStr">
+        <is>
+          <t>0.01:2</t>
+        </is>
+      </c>
+      <c r="AH7" s="8" t="inlineStr"/>
+      <c r="AI7" s="8" t="inlineStr"/>
+      <c r="AJ7" s="8" t="inlineStr"/>
+      <c r="AK7" s="8" t="inlineStr"/>
+      <c r="AL7" s="8" t="inlineStr"/>
+      <c r="AM7" s="8" t="inlineStr"/>
+      <c r="AN7" s="8" t="inlineStr"/>
+      <c r="AO7" s="8" t="inlineStr"/>
+      <c r="AP7" s="8" t="inlineStr"/>
       <c r="AS7" t="inlineStr">
         <is>
           <t>Analyser Mode</t>
@@ -1048,6 +1481,101 @@
       <c r="G8" t="n">
         <v>679936</v>
       </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Y8" s="6" t="inlineStr">
+        <is>
+          <t>S2p .</t>
+        </is>
+      </c>
+      <c r="Z8" s="6" t="inlineStr">
+        <is>
+          <t>161.86</t>
+        </is>
+      </c>
+      <c r="AA8" s="6" t="inlineStr">
+        <is>
+          <t>76896.06</t>
+        </is>
+      </c>
+      <c r="AB8" s="6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AC8" s="6" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="AD8" s="6" t="inlineStr">
+        <is>
+          <t>231415.65</t>
+        </is>
+      </c>
+      <c r="AE8" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AF8" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AG8" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AH8" s="6" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="AI8" s="6" t="inlineStr">
+        <is>
+          <t>91.82</t>
+        </is>
+      </c>
+      <c r="AJ8" s="6" t="inlineStr">
+        <is>
+          <t>-771.00</t>
+        </is>
+      </c>
+      <c r="AK8" s="6" t="inlineStr">
+        <is>
+          <t>Unfitted</t>
+        </is>
+      </c>
+      <c r="AL8" s="6" t="inlineStr">
+        <is>
+          <t>U2-Tougaard</t>
+        </is>
+      </c>
+      <c r="AM8" s="6" t="inlineStr">
+        <is>
+          <t>151.36</t>
+        </is>
+      </c>
+      <c r="AN8" s="6" t="inlineStr">
+        <is>
+          <t>175.86</t>
+        </is>
+      </c>
+      <c r="AO8" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AP8" s="6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
       <c r="AS8" t="inlineStr">
         <is>
           <t>Energy Step Size</t>
@@ -1072,6 +1600,57 @@
       <c r="G9" t="n">
         <v>682097</v>
       </c>
+      <c r="X9" s="7" t="inlineStr"/>
+      <c r="Y9" s="8" t="inlineStr"/>
+      <c r="Z9" s="8" t="inlineStr">
+        <is>
+          <t>-9.64:1350.36</t>
+        </is>
+      </c>
+      <c r="AA9" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AB9" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3.7</t>
+        </is>
+      </c>
+      <c r="AC9" s="8" t="inlineStr">
+        <is>
+          <t>5:80</t>
+        </is>
+      </c>
+      <c r="AD9" s="8" t="inlineStr">
+        <is>
+          <t>1:1e7</t>
+        </is>
+      </c>
+      <c r="AE9" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AF9" s="8" t="inlineStr">
+        <is>
+          <t>0.3:3</t>
+        </is>
+      </c>
+      <c r="AG9" s="8" t="inlineStr">
+        <is>
+          <t>0.01:2</t>
+        </is>
+      </c>
+      <c r="AH9" s="8" t="inlineStr"/>
+      <c r="AI9" s="8" t="inlineStr"/>
+      <c r="AJ9" s="8" t="inlineStr"/>
+      <c r="AK9" s="8" t="inlineStr"/>
+      <c r="AL9" s="8" t="inlineStr"/>
+      <c r="AM9" s="8" t="inlineStr"/>
+      <c r="AN9" s="8" t="inlineStr"/>
+      <c r="AO9" s="8" t="inlineStr"/>
+      <c r="AP9" s="8" t="inlineStr"/>
       <c r="AS9" t="inlineStr">
         <is>
           <t>Number of Energy Steps</t>
@@ -1096,6 +1675,11 @@
       <c r="G10" t="n">
         <v>694729</v>
       </c>
+      <c r="X10" s="4" t="inlineStr">
+        <is>
+          <t>Please cite G.Kerherve, W.Skinner, J.Hochhaus, et al., Surface and Interface Analysis (2025): 1–12, https://doi.org/10.1002/sia.70032</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -11972,7 +12556,7 @@
         <v>957.86</v>
       </c>
       <c r="G787" t="n">
-        <v>231857</v>
+        <v>230255.4478291747</v>
       </c>
     </row>
     <row r="788">
@@ -11986,7 +12570,7 @@
         <v>957.36</v>
       </c>
       <c r="G788" t="n">
-        <v>226152</v>
+        <v>229975.682504905</v>
       </c>
     </row>
     <row r="789">
@@ -12000,7 +12584,7 @@
         <v>956.86</v>
       </c>
       <c r="G789" t="n">
-        <v>226643</v>
+        <v>229690.9644554636</v>
       </c>
     </row>
     <row r="790">
@@ -12014,7 +12598,7 @@
         <v>956.36</v>
       </c>
       <c r="G790" t="n">
-        <v>228283</v>
+        <v>229401.8929617121</v>
       </c>
     </row>
     <row r="791">
@@ -12028,7 +12612,7 @@
         <v>955.86</v>
       </c>
       <c r="G791" t="n">
-        <v>235499</v>
+        <v>229109.9929495947</v>
       </c>
     </row>
     <row r="792">
@@ -12042,7 +12626,7 @@
         <v>955.36</v>
       </c>
       <c r="G792" t="n">
-        <v>234572</v>
+        <v>228821.2413070076</v>
       </c>
     </row>
     <row r="793">
@@ -12056,7 +12640,7 @@
         <v>954.86</v>
       </c>
       <c r="G793" t="n">
-        <v>237866</v>
+        <v>228535.1179971534</v>
       </c>
     </row>
     <row r="794">
@@ -12070,7 +12654,7 @@
         <v>954.36</v>
       </c>
       <c r="G794" t="n">
-        <v>242046</v>
+        <v>228254.4639778595</v>
       </c>
     </row>
     <row r="795">
@@ -12084,7 +12668,7 @@
         <v>953.86</v>
       </c>
       <c r="G795" t="n">
-        <v>243189</v>
+        <v>227982.8168439639</v>
       </c>
     </row>
     <row r="796">
@@ -12098,7 +12682,7 @@
         <v>953.36</v>
       </c>
       <c r="G796" t="n">
-        <v>249740</v>
+        <v>227721.2764657282</v>
       </c>
     </row>
     <row r="797">
@@ -12112,7 +12696,7 @@
         <v>952.86</v>
       </c>
       <c r="G797" t="n">
-        <v>255951</v>
+        <v>227475.2356623198</v>
       </c>
     </row>
     <row r="798">
@@ -12126,7 +12710,7 @@
         <v>952.36</v>
       </c>
       <c r="G798" t="n">
-        <v>258055</v>
+        <v>227249.7876291111</v>
       </c>
     </row>
     <row r="799">
@@ -12140,7 +12724,7 @@
         <v>951.86</v>
       </c>
       <c r="G799" t="n">
-        <v>251597</v>
+        <v>227046.7134075818</v>
       </c>
     </row>
     <row r="800">
@@ -12154,7 +12738,7 @@
         <v>951.36</v>
       </c>
       <c r="G800" t="n">
-        <v>248715</v>
+        <v>226860.9270376298</v>
       </c>
     </row>
     <row r="801">
@@ -12168,7 +12752,7 @@
         <v>950.86</v>
       </c>
       <c r="G801" t="n">
-        <v>237443</v>
+        <v>226690.1623335193</v>
       </c>
     </row>
     <row r="802">
@@ -12182,7 +12766,7 @@
         <v>950.36</v>
       </c>
       <c r="G802" t="n">
-        <v>234660</v>
+        <v>226525.4375104628</v>
       </c>
     </row>
     <row r="803">
@@ -12196,7 +12780,7 @@
         <v>949.86</v>
       </c>
       <c r="G803" t="n">
-        <v>228176</v>
+        <v>226364.5291477455</v>
       </c>
     </row>
     <row r="804">
@@ -12210,7 +12794,7 @@
         <v>949.36</v>
       </c>
       <c r="G804" t="n">
-        <v>230387</v>
+        <v>226202.2583639919</v>
       </c>
     </row>
     <row r="805">
@@ -12224,7 +12808,7 @@
         <v>948.86</v>
       </c>
       <c r="G805" t="n">
-        <v>226676</v>
+        <v>226040.3838788281</v>
       </c>
     </row>
     <row r="806">
@@ -12238,7 +12822,7 @@
         <v>948.36</v>
       </c>
       <c r="G806" t="n">
-        <v>225811</v>
+        <v>225875.9460809121</v>
       </c>
     </row>
     <row r="807">
@@ -12252,7 +12836,7 @@
         <v>947.86</v>
       </c>
       <c r="G807" t="n">
-        <v>228420</v>
+        <v>225708.2636629358</v>
       </c>
     </row>
     <row r="808">
@@ -12266,7 +12850,7 @@
         <v>947.36</v>
       </c>
       <c r="G808" t="n">
-        <v>227245</v>
+        <v>225539.4364273298</v>
       </c>
     </row>
     <row r="809">
@@ -12280,7 +12864,7 @@
         <v>946.86</v>
       </c>
       <c r="G809" t="n">
-        <v>226554</v>
+        <v>225368.5558388551</v>
       </c>
     </row>
     <row r="810">
@@ -12294,7 +12878,7 @@
         <v>946.36</v>
       </c>
       <c r="G810" t="n">
-        <v>223264</v>
+        <v>225195.1102934463</v>
       </c>
     </row>
     <row r="811">
@@ -12308,7 +12892,7 @@
         <v>945.86</v>
       </c>
       <c r="G811" t="n">
-        <v>220972</v>
+        <v>225016.5290071627</v>
       </c>
     </row>
     <row r="812">
@@ -12322,7 +12906,7 @@
         <v>945.36</v>
       </c>
       <c r="G812" t="n">
-        <v>218807</v>
+        <v>224831.0553446307</v>
       </c>
     </row>
     <row r="813">
@@ -12336,7 +12920,7 @@
         <v>944.86</v>
       </c>
       <c r="G813" t="n">
-        <v>228635</v>
+        <v>224637.0564716924</v>
       </c>
     </row>
     <row r="814">
@@ -12350,7 +12934,7 @@
         <v>944.36</v>
       </c>
       <c r="G814" t="n">
-        <v>221542</v>
+        <v>224442.4874252652</v>
       </c>
     </row>
     <row r="815">
@@ -12364,7 +12948,7 @@
         <v>943.86</v>
       </c>
       <c r="G815" t="n">
-        <v>227029</v>
+        <v>224241.8253709574</v>
       </c>
     </row>
     <row r="816">
@@ -12378,7 +12962,7 @@
         <v>943.36</v>
       </c>
       <c r="G816" t="n">
-        <v>218880</v>
+        <v>224039.6003305707</v>
       </c>
     </row>
     <row r="817">
@@ -12392,7 +12976,7 @@
         <v>942.86</v>
       </c>
       <c r="G817" t="n">
-        <v>220847</v>
+        <v>223829.4865734765</v>
       </c>
     </row>
     <row r="818">
@@ -12406,7 +12990,7 @@
         <v>942.36</v>
       </c>
       <c r="G818" t="n">
-        <v>223198</v>
+        <v>223613.2512167612</v>
       </c>
     </row>
     <row r="819">
@@ -12420,7 +13004,7 @@
         <v>941.86</v>
       </c>
       <c r="G819" t="n">
-        <v>219656</v>
+        <v>223392.9925104662</v>
       </c>
     </row>
     <row r="820">
@@ -12434,7 +13018,7 @@
         <v>941.36</v>
       </c>
       <c r="G820" t="n">
-        <v>219102</v>
+        <v>223166.1319426136</v>
       </c>
     </row>
     <row r="821">
@@ -12448,7 +13032,7 @@
         <v>940.86</v>
       </c>
       <c r="G821" t="n">
-        <v>221564</v>
+        <v>222932.4996324402</v>
       </c>
     </row>
     <row r="822">
@@ -12462,7 +13046,7 @@
         <v>940.36</v>
       </c>
       <c r="G822" t="n">
-        <v>220144</v>
+        <v>222694.3570635168</v>
       </c>
     </row>
     <row r="823">
@@ -12476,7 +13060,7 @@
         <v>939.86</v>
       </c>
       <c r="G823" t="n">
-        <v>222024</v>
+        <v>222450.8934275835</v>
       </c>
     </row>
     <row r="824">
@@ -12490,7 +13074,7 @@
         <v>939.36</v>
       </c>
       <c r="G824" t="n">
-        <v>223253</v>
+        <v>222203.9528626254</v>
       </c>
     </row>
     <row r="825">
@@ -12504,7 +13088,7 @@
         <v>938.86</v>
       </c>
       <c r="G825" t="n">
-        <v>214870</v>
+        <v>221954.8808211021</v>
       </c>
     </row>
     <row r="826">
@@ -12518,7 +13102,7 @@
         <v>938.36</v>
       </c>
       <c r="G826" t="n">
-        <v>218889</v>
+        <v>221697.3769497229</v>
       </c>
     </row>
     <row r="827">
@@ -12532,7 +13116,7 @@
         <v>937.86</v>
       </c>
       <c r="G827" t="n">
-        <v>222877</v>
+        <v>221435.0569146493</v>
       </c>
     </row>
     <row r="828">
@@ -12546,7 +13130,7 @@
         <v>937.36</v>
       </c>
       <c r="G828" t="n">
-        <v>221431</v>
+        <v>221171.5327806161</v>
       </c>
     </row>
     <row r="829">
@@ -12560,7 +13144,7 @@
         <v>936.86</v>
       </c>
       <c r="G829" t="n">
-        <v>220214</v>
+        <v>220906.0980006388</v>
       </c>
     </row>
     <row r="830">
@@ -12574,7 +13158,7 @@
         <v>936.36</v>
       </c>
       <c r="G830" t="n">
-        <v>220959</v>
+        <v>220638.2426508613</v>
       </c>
     </row>
     <row r="831">
@@ -12588,7 +13172,7 @@
         <v>935.86</v>
       </c>
       <c r="G831" t="n">
-        <v>221038</v>
+        <v>220369.0349694178</v>
       </c>
     </row>
     <row r="832">
@@ -12602,7 +13186,7 @@
         <v>935.36</v>
       </c>
       <c r="G832" t="n">
-        <v>228690</v>
+        <v>220099.0230646171</v>
       </c>
     </row>
     <row r="833">
@@ -12616,7 +13200,7 @@
         <v>934.86</v>
       </c>
       <c r="G833" t="n">
-        <v>234333</v>
+        <v>219834.8013045883</v>
       </c>
     </row>
     <row r="834">
@@ -12630,7 +13214,7 @@
         <v>934.36</v>
       </c>
       <c r="G834" t="n">
-        <v>240814</v>
+        <v>219581.3576364148</v>
       </c>
     </row>
     <row r="835">
@@ -12644,7 +13228,7 @@
         <v>933.86</v>
       </c>
       <c r="G835" t="n">
-        <v>257565</v>
+        <v>219344.3329448325</v>
       </c>
     </row>
     <row r="836">
@@ -12658,7 +13242,7 @@
         <v>933.36</v>
       </c>
       <c r="G836" t="n">
-        <v>278220</v>
+        <v>219137.5291797714</v>
       </c>
     </row>
     <row r="837">
@@ -12672,7 +13256,7 @@
         <v>932.86</v>
       </c>
       <c r="G837" t="n">
-        <v>291033</v>
+        <v>218977.8075322972</v>
       </c>
     </row>
     <row r="838">
@@ -12686,7 +13270,7 @@
         <v>932.36</v>
       </c>
       <c r="G838" t="n">
-        <v>283844</v>
+        <v>218875.6918985739</v>
       </c>
     </row>
     <row r="839">
@@ -12700,7 +13284,7 @@
         <v>931.86</v>
       </c>
       <c r="G839" t="n">
-        <v>263834</v>
+        <v>218825.6540614175</v>
       </c>
     </row>
     <row r="840">
@@ -12714,7 +13298,7 @@
         <v>931.36</v>
       </c>
       <c r="G840" t="n">
-        <v>244095</v>
+        <v>218811.8482392106</v>
       </c>
     </row>
     <row r="841">
@@ -12728,7 +13312,7 @@
         <v>930.86</v>
       </c>
       <c r="G841" t="n">
-        <v>231917</v>
+        <v>218818.5773219402</v>
       </c>
     </row>
     <row r="842">
@@ -12742,7 +13326,7 @@
         <v>930.36</v>
       </c>
       <c r="G842" t="n">
-        <v>227383</v>
+        <v>218836.1333226411</v>
       </c>
     </row>
     <row r="843">
@@ -12756,7 +13340,7 @@
         <v>929.86</v>
       </c>
       <c r="G843" t="n">
-        <v>217646</v>
+        <v>218860.8811633684</v>
       </c>
     </row>
     <row r="844">
@@ -12770,7 +13354,7 @@
         <v>929.36</v>
       </c>
       <c r="G844" t="n">
-        <v>222002</v>
+        <v>218885.0228789446</v>
       </c>
     </row>
     <row r="845">
@@ -12784,7 +13368,7 @@
         <v>928.86</v>
       </c>
       <c r="G845" t="n">
-        <v>223030</v>
+        <v>218911.9957798461</v>
       </c>
     </row>
     <row r="846">
@@ -12798,7 +13382,7 @@
         <v>928.36</v>
       </c>
       <c r="G846" t="n">
-        <v>216584</v>
+        <v>218942.5771436312</v>
       </c>
     </row>
     <row r="847">
@@ -12812,7 +13396,7 @@
         <v>927.86</v>
       </c>
       <c r="G847" t="n">
-        <v>219044</v>
+        <v>218971.5774076481</v>
       </c>
     </row>
     <row r="848">
@@ -12826,7 +13410,7 @@
         <v>927.36</v>
       </c>
       <c r="G848" t="n">
-        <v>219550</v>
+        <v>219000.908829698</v>
       </c>
     </row>
     <row r="849">
@@ -12840,7 +13424,7 @@
         <v>926.86</v>
       </c>
       <c r="G849" t="n">
-        <v>214798</v>
+        <v>219030.9238434694</v>
       </c>
     </row>
     <row r="850">
@@ -12854,7 +13438,7 @@
         <v>926.36</v>
       </c>
       <c r="G850" t="n">
-        <v>216046</v>
+        <v>219057.7803672281</v>
       </c>
     </row>
     <row r="851">
@@ -12868,7 +13452,7 @@
         <v>925.86</v>
       </c>
       <c r="G851" t="n">
-        <v>218052</v>
+        <v>219082.4244749444</v>
       </c>
     </row>
     <row r="852">
@@ -12882,7 +13466,7 @@
         <v>925.36</v>
       </c>
       <c r="G852" t="n">
-        <v>219738</v>
+        <v>219106.4095427157</v>
       </c>
     </row>
     <row r="853">
@@ -12896,7 +13480,7 @@
         <v>924.86</v>
       </c>
       <c r="G853" t="n">
-        <v>214298</v>
+        <v>219131.0340756189</v>
       </c>
     </row>
     <row r="854">
@@ -12910,7 +13494,7 @@
         <v>924.36</v>
       </c>
       <c r="G854" t="n">
-        <v>219625</v>
+        <v>219151.9133025262</v>
       </c>
     </row>
     <row r="855">
@@ -12924,7 +13508,7 @@
         <v>923.86</v>
       </c>
       <c r="G855" t="n">
-        <v>216718</v>
+        <v>219173.2526676655</v>
       </c>
     </row>
     <row r="856">
@@ -12938,7 +13522,7 @@
         <v>923.36</v>
       </c>
       <c r="G856" t="n">
-        <v>215242</v>
+        <v>219192.6915416972</v>
       </c>
     </row>
     <row r="857">
@@ -12952,7 +13536,7 @@
         <v>922.86</v>
       </c>
       <c r="G857" t="n">
-        <v>216187</v>
+        <v>219209.0131664526</v>
       </c>
     </row>
     <row r="858">
@@ -12966,7 +13550,7 @@
         <v>922.36</v>
       </c>
       <c r="G858" t="n">
-        <v>216065</v>
+        <v>219222.9362817839</v>
       </c>
     </row>
     <row r="859">
@@ -12980,7 +13564,7 @@
         <v>921.86</v>
       </c>
       <c r="G859" t="n">
-        <v>218868</v>
+        <v>219234.3330819542</v>
       </c>
     </row>
     <row r="860">
@@ -12994,7 +13578,7 @@
         <v>921.36</v>
       </c>
       <c r="G860" t="n">
-        <v>215697</v>
+        <v>219245.412210688</v>
       </c>
     </row>
     <row r="861">
@@ -13008,7 +13592,7 @@
         <v>920.86</v>
       </c>
       <c r="G861" t="n">
-        <v>215440</v>
+        <v>219253.6200098397</v>
       </c>
     </row>
     <row r="862">
@@ -13022,7 +13606,7 @@
         <v>920.36</v>
       </c>
       <c r="G862" t="n">
-        <v>218425</v>
+        <v>219258.7313144449</v>
       </c>
     </row>
     <row r="863">
@@ -13036,7 +13620,7 @@
         <v>919.86</v>
       </c>
       <c r="G863" t="n">
-        <v>218099</v>
+        <v>219263.1114439522</v>
       </c>
     </row>
     <row r="864">
@@ -13050,7 +13634,7 @@
         <v>919.36</v>
       </c>
       <c r="G864" t="n">
-        <v>220274</v>
+        <v>219266.4875086761</v>
       </c>
     </row>
     <row r="865">
@@ -13064,7 +13648,7 @@
         <v>918.86</v>
       </c>
       <c r="G865" t="n">
-        <v>214254</v>
+        <v>219270.5826410957</v>
       </c>
     </row>
     <row r="866">
@@ -13078,7 +13662,7 @@
         <v>918.36</v>
       </c>
       <c r="G866" t="n">
-        <v>214790</v>
+        <v>219270.5854172779</v>
       </c>
     </row>
     <row r="867">
@@ -13092,7 +13676,7 @@
         <v>917.86</v>
       </c>
       <c r="G867" t="n">
-        <v>216892</v>
+        <v>219266.9190683548</v>
       </c>
     </row>
     <row r="868">
@@ -13106,7 +13690,7 @@
         <v>917.36</v>
       </c>
       <c r="G868" t="n">
-        <v>219109</v>
+        <v>219261.2624164073</v>
       </c>
     </row>
     <row r="869">
@@ -13120,7 +13704,7 @@
         <v>916.86</v>
       </c>
       <c r="G869" t="n">
-        <v>218328</v>
+        <v>219255.3900005672</v>
       </c>
     </row>
     <row r="870">
@@ -13134,7 +13718,7 @@
         <v>916.36</v>
       </c>
       <c r="G870" t="n">
-        <v>216141</v>
+        <v>219248.6869700712</v>
       </c>
     </row>
     <row r="871">
@@ -13148,7 +13732,7 @@
         <v>915.86</v>
       </c>
       <c r="G871" t="n">
-        <v>220967</v>
+        <v>219239.4194390388</v>
       </c>
     </row>
     <row r="872">
@@ -13162,7 +13746,7 @@
         <v>915.36</v>
       </c>
       <c r="G872" t="n">
-        <v>219302</v>
+        <v>219231.44976718</v>
       </c>
     </row>
     <row r="873">
@@ -13176,7 +13760,7 @@
         <v>914.86</v>
       </c>
       <c r="G873" t="n">
-        <v>218647</v>
+        <v>219223.4632913757</v>
       </c>
     </row>
     <row r="874">
@@ -13190,7 +13774,7 @@
         <v>914.36</v>
       </c>
       <c r="G874" t="n">
-        <v>218252</v>
+        <v>219214.9509447342</v>
       </c>
     </row>
     <row r="875">
@@ -13204,7 +13788,7 @@
         <v>913.86</v>
       </c>
       <c r="G875" t="n">
-        <v>219284</v>
+        <v>219205.6122135817</v>
       </c>
     </row>
     <row r="876">
@@ -13218,7 +13802,7 @@
         <v>913.36</v>
       </c>
       <c r="G876" t="n">
-        <v>217505</v>
+        <v>219196.2860554375</v>
       </c>
     </row>
     <row r="877">
@@ -13232,7 +13816,7 @@
         <v>912.86</v>
       </c>
       <c r="G877" t="n">
-        <v>222274</v>
+        <v>219185.5705431687</v>
       </c>
     </row>
     <row r="878">
@@ -13246,7 +13830,7 @@
         <v>912.36</v>
       </c>
       <c r="G878" t="n">
-        <v>220170</v>
+        <v>219177.2869348933</v>
       </c>
     </row>
     <row r="879">
@@ -13260,7 +13844,7 @@
         <v>911.86</v>
       </c>
       <c r="G879" t="n">
-        <v>224012</v>
+        <v>219169.7726311036</v>
       </c>
     </row>
     <row r="880">
@@ -13274,7 +13858,7 @@
         <v>911.36</v>
       </c>
       <c r="G880" t="n">
-        <v>216528</v>
+        <v>219166.1042406741</v>
       </c>
     </row>
     <row r="881">
@@ -13288,7 +13872,7 @@
         <v>910.86</v>
       </c>
       <c r="G881" t="n">
-        <v>224433</v>
+        <v>219160.3216632776</v>
       </c>
     </row>
     <row r="882">
@@ -13302,7 +13886,7 @@
         <v>910.36</v>
       </c>
       <c r="G882" t="n">
-        <v>219534</v>
+        <v>219158.7377373057</v>
       </c>
     </row>
     <row r="883">
@@ -13316,7 +13900,7 @@
         <v>909.86</v>
       </c>
       <c r="G883" t="n">
-        <v>220076</v>
+        <v>219157.4495529276</v>
       </c>
     </row>
     <row r="884">
@@ -13330,7 +13914,7 @@
         <v>909.36</v>
       </c>
       <c r="G884" t="n">
-        <v>217019</v>
+        <v>219156.8915672809</v>
       </c>
     </row>
     <row r="885">
@@ -13344,7 +13928,7 @@
         <v>908.86</v>
       </c>
       <c r="G885" t="n">
-        <v>221343</v>
+        <v>219154.6275782297</v>
       </c>
     </row>
     <row r="886">
@@ -13358,7 +13942,7 @@
         <v>908.36</v>
       </c>
       <c r="G886" t="n">
-        <v>221422</v>
+        <v>219154.1090771685</v>
       </c>
     </row>
     <row r="887">
@@ -13372,7 +13956,7 @@
         <v>907.86</v>
       </c>
       <c r="G887" t="n">
-        <v>215917</v>
+        <v>219155.4</v>
       </c>
     </row>
     <row r="888">
@@ -28002,7 +28586,7 @@
         <v>385.36</v>
       </c>
       <c r="G1932" t="n">
-        <v>250054</v>
+        <v>257611.82205375</v>
       </c>
     </row>
     <row r="1933">
@@ -28016,7 +28600,7 @@
         <v>384.86</v>
       </c>
       <c r="G1933" t="n">
-        <v>249145</v>
+        <v>251858.8018015228</v>
       </c>
     </row>
     <row r="1934">
@@ -28030,7 +28614,7 @@
         <v>384.36</v>
       </c>
       <c r="G1934" t="n">
-        <v>246228</v>
+        <v>246013.1248913919</v>
       </c>
     </row>
     <row r="1935">
@@ -28044,7 +28628,7 @@
         <v>383.86</v>
       </c>
       <c r="G1935" t="n">
-        <v>242508</v>
+        <v>240075.5756928036</v>
       </c>
     </row>
     <row r="1936">
@@ -28058,7 +28642,7 @@
         <v>383.36</v>
       </c>
       <c r="G1936" t="n">
-        <v>241671</v>
+        <v>234046.6863599665</v>
       </c>
     </row>
     <row r="1937">
@@ -28072,7 +28656,7 @@
         <v>382.86</v>
       </c>
       <c r="G1937" t="n">
-        <v>232209</v>
+        <v>227929.7958787921</v>
       </c>
     </row>
     <row r="1938">
@@ -28086,7 +28670,7 @@
         <v>382.36</v>
       </c>
       <c r="G1938" t="n">
-        <v>227834</v>
+        <v>221721.5541315122</v>
       </c>
     </row>
     <row r="1939">
@@ -28100,7 +28684,7 @@
         <v>381.86</v>
       </c>
       <c r="G1939" t="n">
-        <v>226759</v>
+        <v>215423.2661636196</v>
       </c>
     </row>
     <row r="1940">
@@ -28114,7 +28698,7 @@
         <v>381.36</v>
       </c>
       <c r="G1940" t="n">
-        <v>219048</v>
+        <v>209039.4258355455</v>
       </c>
     </row>
     <row r="1941">
@@ -28128,7 +28712,7 @@
         <v>380.86</v>
       </c>
       <c r="G1941" t="n">
-        <v>219041</v>
+        <v>202569.5117504299</v>
       </c>
     </row>
     <row r="1942">
@@ -28142,7 +28726,7 @@
         <v>380.36</v>
       </c>
       <c r="G1942" t="n">
-        <v>210910</v>
+        <v>196019.8401711445</v>
       </c>
     </row>
     <row r="1943">
@@ -28156,7 +28740,7 @@
         <v>379.86</v>
       </c>
       <c r="G1943" t="n">
-        <v>208975</v>
+        <v>189390.4877052071</v>
       </c>
     </row>
     <row r="1944">
@@ -28170,7 +28754,7 @@
         <v>379.36</v>
       </c>
       <c r="G1944" t="n">
-        <v>209303</v>
+        <v>182687.122640493</v>
       </c>
     </row>
     <row r="1945">
@@ -28184,7 +28768,7 @@
         <v>378.86</v>
       </c>
       <c r="G1945" t="n">
-        <v>200160</v>
+        <v>175917.7487088142</v>
       </c>
     </row>
     <row r="1946">
@@ -28198,7 +28782,7 @@
         <v>378.36</v>
       </c>
       <c r="G1946" t="n">
-        <v>201327</v>
+        <v>169082.9994670442</v>
       </c>
     </row>
     <row r="1947">
@@ -28212,7 +28796,7 @@
         <v>377.86</v>
       </c>
       <c r="G1947" t="n">
-        <v>201476</v>
+        <v>162192.4721331585</v>
       </c>
     </row>
     <row r="1948">
@@ -28226,7 +28810,7 @@
         <v>377.36</v>
       </c>
       <c r="G1948" t="n">
-        <v>202149</v>
+        <v>155255.3496875801</v>
       </c>
     </row>
     <row r="1949">
@@ -28240,7 +28824,7 @@
         <v>376.86</v>
       </c>
       <c r="G1949" t="n">
-        <v>207126</v>
+        <v>148281.6507139113</v>
       </c>
     </row>
     <row r="1950">
@@ -28254,7 +28838,7 @@
         <v>376.36</v>
       </c>
       <c r="G1950" t="n">
-        <v>236850</v>
+        <v>141285.323721994</v>
       </c>
     </row>
     <row r="1951">
@@ -28268,7 +28852,7 @@
         <v>375.86</v>
       </c>
       <c r="G1951" t="n">
-        <v>328758</v>
+        <v>134301.0939995503</v>
       </c>
     </row>
     <row r="1952">
@@ -28282,7 +28866,7 @@
         <v>375.36</v>
       </c>
       <c r="G1952" t="n">
-        <v>538735</v>
+        <v>127415.3057226009</v>
       </c>
     </row>
     <row r="1953">
@@ -28296,7 +28880,7 @@
         <v>374.86</v>
       </c>
       <c r="G1953" t="n">
-        <v>836940</v>
+        <v>120811.9041387422</v>
       </c>
     </row>
     <row r="1954">
@@ -28310,7 +28894,7 @@
         <v>374.36</v>
       </c>
       <c r="G1954" t="n">
-        <v>962084</v>
+        <v>114747.4368633898</v>
       </c>
     </row>
     <row r="1955">
@@ -28324,7 +28908,7 @@
         <v>373.86</v>
       </c>
       <c r="G1955" t="n">
-        <v>792622</v>
+        <v>109334.7687338449</v>
       </c>
     </row>
     <row r="1956">
@@ -28338,7 +28922,7 @@
         <v>373.36</v>
       </c>
       <c r="G1956" t="n">
-        <v>497313</v>
+        <v>104442.4746046467</v>
       </c>
     </row>
     <row r="1957">
@@ -28352,7 +28936,7 @@
         <v>372.86</v>
       </c>
       <c r="G1957" t="n">
-        <v>296006</v>
+        <v>99834.44217758137</v>
       </c>
     </row>
     <row r="1958">
@@ -28366,7 +28950,7 @@
         <v>372.36</v>
       </c>
       <c r="G1958" t="n">
-        <v>209684</v>
+        <v>95351.86215894102</v>
       </c>
     </row>
     <row r="1959">
@@ -28380,7 +28964,7 @@
         <v>371.86</v>
       </c>
       <c r="G1959" t="n">
-        <v>185447</v>
+        <v>90930.83333522863</v>
       </c>
     </row>
     <row r="1960">
@@ -28394,7 +28978,7 @@
         <v>371.36</v>
       </c>
       <c r="G1960" t="n">
-        <v>174778</v>
+        <v>86558.77352647248</v>
       </c>
     </row>
     <row r="1961">
@@ -28408,7 +28992,7 @@
         <v>370.86</v>
       </c>
       <c r="G1961" t="n">
-        <v>181581</v>
+        <v>82234.35581729081</v>
       </c>
     </row>
     <row r="1962">
@@ -28422,7 +29006,7 @@
         <v>370.36</v>
       </c>
       <c r="G1962" t="n">
-        <v>222072</v>
+        <v>77970.7179241346</v>
       </c>
     </row>
     <row r="1963">
@@ -28436,7 +29020,7 @@
         <v>369.86</v>
       </c>
       <c r="G1963" t="n">
-        <v>352502</v>
+        <v>73808.81284983321</v>
       </c>
     </row>
     <row r="1964">
@@ -28450,7 +29034,7 @@
         <v>369.36</v>
       </c>
       <c r="G1964" t="n">
-        <v>662825</v>
+        <v>69863.77318099728</v>
       </c>
     </row>
     <row r="1965">
@@ -28464,7 +29048,7 @@
         <v>368.86</v>
       </c>
       <c r="G1965" t="n">
-        <v>1090460</v>
+        <v>66398.97519218204</v>
       </c>
     </row>
     <row r="1966">
@@ -28478,7 +29062,7 @@
         <v>368.36</v>
       </c>
       <c r="G1966" t="n">
-        <v>1274240</v>
+        <v>63773.85393989091</v>
       </c>
     </row>
     <row r="1967">
@@ -28492,7 +29076,7 @@
         <v>367.86</v>
       </c>
       <c r="G1967" t="n">
-        <v>1007410</v>
+        <v>62144.94214137104</v>
       </c>
     </row>
     <row r="1968">
@@ -28506,7 +29090,7 @@
         <v>367.36</v>
       </c>
       <c r="G1968" t="n">
-        <v>581086</v>
+        <v>61294.81240308805</v>
       </c>
     </row>
     <row r="1969">
@@ -28520,7 +29104,7 @@
         <v>366.86</v>
       </c>
       <c r="G1969" t="n">
-        <v>285315</v>
+        <v>60872.89943246636</v>
       </c>
     </row>
     <row r="1970">
@@ -28534,7 +29118,7 @@
         <v>366.36</v>
       </c>
       <c r="G1970" t="n">
-        <v>164747</v>
+        <v>60635.68605372321</v>
       </c>
     </row>
     <row r="1971">
@@ -28548,7 +29132,7 @@
         <v>365.86</v>
       </c>
       <c r="G1971" t="n">
-        <v>119821</v>
+        <v>60484.02200712434</v>
       </c>
     </row>
     <row r="1972">
@@ -28562,7 +29146,7 @@
         <v>365.36</v>
       </c>
       <c r="G1972" t="n">
-        <v>98389.2</v>
+        <v>60381.0760254657</v>
       </c>
     </row>
     <row r="1973">
@@ -28576,7 +29160,7 @@
         <v>364.86</v>
       </c>
       <c r="G1973" t="n">
-        <v>88624.89999999999</v>
+        <v>60309.33330471108</v>
       </c>
     </row>
     <row r="1974">
@@ -28590,7 +29174,7 @@
         <v>364.36</v>
       </c>
       <c r="G1974" t="n">
-        <v>80445.3</v>
+        <v>60260.85926220854</v>
       </c>
     </row>
     <row r="1975">
@@ -28604,7 +29188,7 @@
         <v>363.86</v>
       </c>
       <c r="G1975" t="n">
-        <v>71506</v>
+        <v>60228.98625516296</v>
       </c>
     </row>
     <row r="1976">
@@ -28618,7 +29202,7 @@
         <v>363.36</v>
       </c>
       <c r="G1976" t="n">
-        <v>72048.3</v>
+        <v>60206.38926248695</v>
       </c>
     </row>
     <row r="1977">
@@ -28632,7 +29216,7 @@
         <v>362.86</v>
       </c>
       <c r="G1977" t="n">
-        <v>67678.5</v>
+        <v>60193.55740704945</v>
       </c>
     </row>
     <row r="1978">
@@ -28646,7 +29230,7 @@
         <v>362.36</v>
       </c>
       <c r="G1978" t="n">
-        <v>66815.89999999999</v>
+        <v>60186.90515728714</v>
       </c>
     </row>
     <row r="1979">
@@ -28660,7 +29244,7 @@
         <v>361.86</v>
       </c>
       <c r="G1979" t="n">
-        <v>62178.4</v>
+        <v>60185.7323251182</v>
       </c>
     </row>
     <row r="1980">
@@ -28674,7 +29258,7 @@
         <v>361.36</v>
       </c>
       <c r="G1980" t="n">
-        <v>62072.4</v>
+        <v>60186.21100443916</v>
       </c>
     </row>
     <row r="1981">
@@ -28688,7 +29272,7 @@
         <v>360.86</v>
       </c>
       <c r="G1981" t="n">
-        <v>60355</v>
+        <v>60188.2528250251</v>
       </c>
     </row>
     <row r="1982">
@@ -28702,7 +29286,7 @@
         <v>360.36</v>
       </c>
       <c r="G1982" t="n">
-        <v>58931.6</v>
+        <v>60190.43567900068</v>
       </c>
     </row>
     <row r="1983">
@@ -28716,7 +29300,7 @@
         <v>359.86</v>
       </c>
       <c r="G1983" t="n">
-        <v>57420.5</v>
+        <v>60191.58</v>
       </c>
     </row>
     <row r="1984">
@@ -30340,7 +30924,7 @@
         <v>301.86</v>
       </c>
       <c r="G2099" t="n">
-        <v>56346</v>
+        <v>57832.00491892958</v>
       </c>
     </row>
     <row r="2100">
@@ -30354,7 +30938,7 @@
         <v>301.36</v>
       </c>
       <c r="G2100" t="n">
-        <v>59298.2</v>
+        <v>57818.7869776965</v>
       </c>
     </row>
     <row r="2101">
@@ -30368,7 +30952,7 @@
         <v>300.86</v>
       </c>
       <c r="G2101" t="n">
-        <v>56971.5</v>
+        <v>57804.90754733526</v>
       </c>
     </row>
     <row r="2102">
@@ -30382,7 +30966,7 @@
         <v>300.36</v>
       </c>
       <c r="G2102" t="n">
-        <v>58135</v>
+        <v>57790.01955143156</v>
       </c>
     </row>
     <row r="2103">
@@ -30396,7 +30980,7 @@
         <v>299.86</v>
       </c>
       <c r="G2103" t="n">
-        <v>58269.3</v>
+        <v>57774.28215577688</v>
       </c>
     </row>
     <row r="2104">
@@ -30410,7 +30994,7 @@
         <v>299.36</v>
       </c>
       <c r="G2104" t="n">
-        <v>56699.6</v>
+        <v>57757.70789763954</v>
       </c>
     </row>
     <row r="2105">
@@ -30424,7 +31008,7 @@
         <v>298.86</v>
       </c>
       <c r="G2105" t="n">
-        <v>58857.5</v>
+        <v>57740.0653315392</v>
       </c>
     </row>
     <row r="2106">
@@ -30438,7 +31022,7 @@
         <v>298.36</v>
       </c>
       <c r="G2106" t="n">
-        <v>58117.6</v>
+        <v>57721.66402407925</v>
       </c>
     </row>
     <row r="2107">
@@ -30452,7 +31036,7 @@
         <v>297.86</v>
       </c>
       <c r="G2107" t="n">
-        <v>57068</v>
+        <v>57702.39725083807</v>
       </c>
     </row>
     <row r="2108">
@@ -30466,7 +31050,7 @@
         <v>297.36</v>
       </c>
       <c r="G2108" t="n">
-        <v>58401.5</v>
+        <v>57682.11609146292</v>
       </c>
     </row>
     <row r="2109">
@@ -30480,7 +31064,7 @@
         <v>296.86</v>
       </c>
       <c r="G2109" t="n">
-        <v>56615.1</v>
+        <v>57661.01871856016</v>
       </c>
     </row>
     <row r="2110">
@@ -30494,7 +31078,7 @@
         <v>296.36</v>
       </c>
       <c r="G2110" t="n">
-        <v>56499</v>
+        <v>57638.85538511549</v>
       </c>
     </row>
     <row r="2111">
@@ -30508,7 +31092,7 @@
         <v>295.86</v>
       </c>
       <c r="G2111" t="n">
-        <v>57470</v>
+        <v>57615.62079729734</v>
       </c>
     </row>
     <row r="2112">
@@ -30522,7 +31106,7 @@
         <v>295.36</v>
       </c>
       <c r="G2112" t="n">
-        <v>57492.5</v>
+        <v>57591.4699897061</v>
       </c>
     </row>
     <row r="2113">
@@ -30536,7 +31120,7 @@
         <v>294.86</v>
       </c>
       <c r="G2113" t="n">
-        <v>56211</v>
+        <v>57566.42413782817</v>
       </c>
     </row>
     <row r="2114">
@@ -30550,7 +31134,7 @@
         <v>294.36</v>
       </c>
       <c r="G2114" t="n">
-        <v>55312.5</v>
+        <v>57540.31924900619</v>
       </c>
     </row>
     <row r="2115">
@@ -30564,7 +31148,7 @@
         <v>293.86</v>
       </c>
       <c r="G2115" t="n">
-        <v>58194.5</v>
+        <v>57513.05016338649</v>
       </c>
     </row>
     <row r="2116">
@@ -30578,7 +31162,7 @@
         <v>293.36</v>
       </c>
       <c r="G2116" t="n">
-        <v>59521.7</v>
+        <v>57485.06146936574</v>
       </c>
     </row>
     <row r="2117">
@@ -30592,7 +31176,7 @@
         <v>292.86</v>
       </c>
       <c r="G2117" t="n">
-        <v>58226.9</v>
+        <v>57456.57618377859</v>
       </c>
     </row>
     <row r="2118">
@@ -30606,7 +31190,7 @@
         <v>292.36</v>
       </c>
       <c r="G2118" t="n">
-        <v>58282.1</v>
+        <v>57427.44123427933</v>
       </c>
     </row>
     <row r="2119">
@@ -30620,7 +31204,7 @@
         <v>291.86</v>
       </c>
       <c r="G2119" t="n">
-        <v>57270.3</v>
+        <v>57397.70139077914</v>
       </c>
     </row>
     <row r="2120">
@@ -30634,7 +31218,7 @@
         <v>291.36</v>
       </c>
       <c r="G2120" t="n">
-        <v>55852.5</v>
+        <v>57367.25010265753</v>
       </c>
     </row>
     <row r="2121">
@@ -30648,7 +31232,7 @@
         <v>290.86</v>
       </c>
       <c r="G2121" t="n">
-        <v>57627.4</v>
+        <v>57335.92513101096</v>
       </c>
     </row>
     <row r="2122">
@@ -30662,7 +31246,7 @@
         <v>290.36</v>
       </c>
       <c r="G2122" t="n">
-        <v>59593.5</v>
+        <v>57304.02853810757</v>
       </c>
     </row>
     <row r="2123">
@@ -30676,7 +31260,7 @@
         <v>289.86</v>
       </c>
       <c r="G2123" t="n">
-        <v>58304.9</v>
+        <v>57271.89259240325</v>
       </c>
     </row>
     <row r="2124">
@@ -30690,7 +31274,7 @@
         <v>289.36</v>
       </c>
       <c r="G2124" t="n">
-        <v>57235.2</v>
+        <v>57239.3814217317</v>
       </c>
     </row>
     <row r="2125">
@@ -30704,7 +31288,7 @@
         <v>288.86</v>
       </c>
       <c r="G2125" t="n">
-        <v>57212.3</v>
+        <v>57206.39284225334</v>
       </c>
     </row>
     <row r="2126">
@@ -30718,7 +31302,7 @@
         <v>288.36</v>
       </c>
       <c r="G2126" t="n">
-        <v>59971.3</v>
+        <v>57172.97801257718</v>
       </c>
     </row>
     <row r="2127">
@@ -30732,7 +31316,7 @@
         <v>287.86</v>
       </c>
       <c r="G2127" t="n">
-        <v>60634.9</v>
+        <v>57139.59181531079</v>
       </c>
     </row>
     <row r="2128">
@@ -30746,7 +31330,7 @@
         <v>287.36</v>
       </c>
       <c r="G2128" t="n">
-        <v>62720.4</v>
+        <v>57106.38750714704</v>
       </c>
     </row>
     <row r="2129">
@@ -30760,7 +31344,7 @@
         <v>286.86</v>
       </c>
       <c r="G2129" t="n">
-        <v>63224.1</v>
+        <v>57073.72428339467</v>
       </c>
     </row>
     <row r="2130">
@@ -30774,7 +31358,7 @@
         <v>286.36</v>
       </c>
       <c r="G2130" t="n">
-        <v>71656.2</v>
+        <v>57041.73267720759</v>
       </c>
     </row>
     <row r="2131">
@@ -30788,7 +31372,7 @@
         <v>285.86</v>
       </c>
       <c r="G2131" t="n">
-        <v>83552.5</v>
+        <v>57011.6876666013</v>
       </c>
     </row>
     <row r="2132">
@@ -30802,7 +31386,7 @@
         <v>285.36</v>
       </c>
       <c r="G2132" t="n">
-        <v>98431.10000000001</v>
+        <v>56985.36146652348</v>
       </c>
     </row>
     <row r="2133">
@@ -30816,7 +31400,7 @@
         <v>284.86</v>
       </c>
       <c r="G2133" t="n">
-        <v>105111</v>
+        <v>56964.95055477457</v>
       </c>
     </row>
     <row r="2134">
@@ -30830,7 +31414,7 @@
         <v>284.36</v>
       </c>
       <c r="G2134" t="n">
-        <v>106438</v>
+        <v>56951.45674332241</v>
       </c>
     </row>
     <row r="2135">
@@ -30844,7 +31428,7 @@
         <v>283.86</v>
       </c>
       <c r="G2135" t="n">
-        <v>84943.3</v>
+        <v>56945.09624918024</v>
       </c>
     </row>
     <row r="2136">
@@ -30858,7 +31442,7 @@
         <v>283.36</v>
       </c>
       <c r="G2136" t="n">
-        <v>69974.39999999999</v>
+        <v>56942.77633670284</v>
       </c>
     </row>
     <row r="2137">
@@ -30872,7 +31456,7 @@
         <v>282.86</v>
       </c>
       <c r="G2137" t="n">
-        <v>60256.9</v>
+        <v>56942.33938208731</v>
       </c>
     </row>
     <row r="2138">
@@ -30886,7 +31470,7 @@
         <v>282.36</v>
       </c>
       <c r="G2138" t="n">
-        <v>58202.5</v>
+        <v>56942.3827454958</v>
       </c>
     </row>
     <row r="2139">
@@ -30900,7 +31484,7 @@
         <v>281.86</v>
       </c>
       <c r="G2139" t="n">
-        <v>57549.3</v>
+        <v>56942.60963280621</v>
       </c>
     </row>
     <row r="2140">
@@ -30914,7 +31498,7 @@
         <v>281.36</v>
       </c>
       <c r="G2140" t="n">
-        <v>55887.3</v>
+        <v>56942.92527504488</v>
       </c>
     </row>
     <row r="2141">
@@ -30928,7 +31512,7 @@
         <v>280.86</v>
       </c>
       <c r="G2141" t="n">
-        <v>59102.2</v>
+        <v>56943.08904314359</v>
       </c>
     </row>
     <row r="2142">
@@ -30942,7 +31526,7 @@
         <v>280.36</v>
       </c>
       <c r="G2142" t="n">
-        <v>56773.9</v>
+        <v>56943.56491911272</v>
       </c>
     </row>
     <row r="2143">
@@ -30956,7 +31540,7 @@
         <v>279.86</v>
       </c>
       <c r="G2143" t="n">
-        <v>55453.1</v>
+        <v>56944.01574856164</v>
       </c>
     </row>
     <row r="2144">
@@ -30970,7 +31554,7 @@
         <v>279.36</v>
       </c>
       <c r="G2144" t="n">
-        <v>55157</v>
+        <v>56944.24993011056</v>
       </c>
     </row>
     <row r="2145">
@@ -30984,7 +31568,7 @@
         <v>278.86</v>
       </c>
       <c r="G2145" t="n">
-        <v>55519.9</v>
+        <v>56944.22425150206</v>
       </c>
     </row>
     <row r="2146">
@@ -30998,7 +31582,7 @@
         <v>278.36</v>
       </c>
       <c r="G2146" t="n">
-        <v>58016.5</v>
+        <v>56943.99115431646</v>
       </c>
     </row>
     <row r="2147">
@@ -31012,7 +31596,7 @@
         <v>277.86</v>
       </c>
       <c r="G2147" t="n">
-        <v>57357.6</v>
+        <v>56943.91161891146</v>
       </c>
     </row>
     <row r="2148">
@@ -31026,7 +31610,7 @@
         <v>277.36</v>
       </c>
       <c r="G2148" t="n">
-        <v>56604.6</v>
+        <v>56943.89062270369</v>
       </c>
     </row>
     <row r="2149">
@@ -31040,7 +31624,7 @@
         <v>276.86</v>
       </c>
       <c r="G2149" t="n">
-        <v>54569</v>
+        <v>56943.81944975303</v>
       </c>
     </row>
     <row r="2150">
@@ -31054,7 +31638,7 @@
         <v>276.36</v>
       </c>
       <c r="G2150" t="n">
-        <v>57422.9</v>
+        <v>56943.4042423105</v>
       </c>
     </row>
     <row r="2151">
@@ -31068,7 +31652,7 @@
         <v>275.86</v>
       </c>
       <c r="G2151" t="n">
-        <v>58541.6</v>
+        <v>56943.05792973386</v>
       </c>
     </row>
     <row r="2152">
@@ -31082,7 +31666,7 @@
         <v>275.36</v>
       </c>
       <c r="G2152" t="n">
-        <v>58411.5</v>
+        <v>56942.9427140429</v>
       </c>
     </row>
     <row r="2153">
@@ -31096,7 +31680,7 @@
         <v>274.86</v>
       </c>
       <c r="G2153" t="n">
-        <v>56002</v>
+        <v>56943.04001957657</v>
       </c>
     </row>
     <row r="2154">
@@ -31110,7 +31694,7 @@
         <v>274.36</v>
       </c>
       <c r="G2154" t="n">
-        <v>57790.7</v>
+        <v>56943.00168393909</v>
       </c>
     </row>
     <row r="2155">
@@ -31124,7 +31708,7 @@
         <v>273.86</v>
       </c>
       <c r="G2155" t="n">
-        <v>57145.8</v>
+        <v>56943.08610802807</v>
       </c>
     </row>
     <row r="2156">
@@ -31138,7 +31722,7 @@
         <v>273.36</v>
       </c>
       <c r="G2156" t="n">
-        <v>55366</v>
+        <v>56943.2</v>
       </c>
     </row>
     <row r="2157">
@@ -33868,7 +34452,7 @@
         <v>175.86</v>
       </c>
       <c r="G2351" t="n">
-        <v>59011.9</v>
+        <v>60047.33119020698</v>
       </c>
     </row>
     <row r="2352">
@@ -33882,7 +34466,7 @@
         <v>175.36</v>
       </c>
       <c r="G2352" t="n">
-        <v>57629.3</v>
+        <v>59719.96089875002</v>
       </c>
     </row>
     <row r="2353">
@@ -33896,7 +34480,7 @@
         <v>174.86</v>
       </c>
       <c r="G2353" t="n">
-        <v>60440.1</v>
+        <v>59386.10082778829</v>
       </c>
     </row>
     <row r="2354">
@@ -33910,7 +34494,7 @@
         <v>174.36</v>
       </c>
       <c r="G2354" t="n">
-        <v>59374.4</v>
+        <v>59048.51634541781</v>
       </c>
     </row>
     <row r="2355">
@@ -33924,7 +34508,7 @@
         <v>173.86</v>
       </c>
       <c r="G2355" t="n">
-        <v>60452.7</v>
+        <v>58706.47908818549</v>
       </c>
     </row>
     <row r="2356">
@@ -33938,7 +34522,7 @@
         <v>173.36</v>
       </c>
       <c r="G2356" t="n">
-        <v>58686.1</v>
+        <v>58361.23070234242</v>
       </c>
     </row>
     <row r="2357">
@@ -33952,7 +34536,7 @@
         <v>172.86</v>
       </c>
       <c r="G2357" t="n">
-        <v>55623.6</v>
+        <v>58011.45567761246</v>
       </c>
     </row>
     <row r="2358">
@@ -33966,7 +34550,7 @@
         <v>172.36</v>
       </c>
       <c r="G2358" t="n">
-        <v>59014.4</v>
+        <v>57654.68964902534</v>
       </c>
     </row>
     <row r="2359">
@@ -33980,7 +34564,7 @@
         <v>171.86</v>
       </c>
       <c r="G2359" t="n">
-        <v>56887.5</v>
+        <v>57294.35423293938</v>
       </c>
     </row>
     <row r="2360">
@@ -33994,7 +34578,7 @@
         <v>171.36</v>
       </c>
       <c r="G2360" t="n">
-        <v>56995.5</v>
+        <v>56928.89171733696</v>
       </c>
     </row>
     <row r="2361">
@@ -34008,7 +34592,7 @@
         <v>170.86</v>
       </c>
       <c r="G2361" t="n">
-        <v>58258.8</v>
+        <v>56558.80107846852</v>
       </c>
     </row>
     <row r="2362">
@@ -34022,7 +34606,7 @@
         <v>170.36</v>
       </c>
       <c r="G2362" t="n">
-        <v>57358.4</v>
+        <v>56185.65793149803</v>
       </c>
     </row>
     <row r="2363">
@@ -34036,7 +34620,7 @@
         <v>169.86</v>
       </c>
       <c r="G2363" t="n">
-        <v>58015.8</v>
+        <v>55809.10088902962</v>
       </c>
     </row>
     <row r="2364">
@@ -34050,7 +34634,7 @@
         <v>169.36</v>
       </c>
       <c r="G2364" t="n">
-        <v>59164.5</v>
+        <v>55430.20813447101</v>
       </c>
     </row>
     <row r="2365">
@@ -34064,7 +34648,7 @@
         <v>168.86</v>
       </c>
       <c r="G2365" t="n">
-        <v>59818.2</v>
+        <v>55050.52775869458</v>
       </c>
     </row>
     <row r="2366">
@@ -34078,7 +34662,7 @@
         <v>168.36</v>
       </c>
       <c r="G2366" t="n">
-        <v>56471</v>
+        <v>54671.17984233125</v>
       </c>
     </row>
     <row r="2367">
@@ -34092,7 +34676,7 @@
         <v>167.86</v>
       </c>
       <c r="G2367" t="n">
-        <v>57469.9</v>
+        <v>54289.67350509933</v>
       </c>
     </row>
     <row r="2368">
@@ -34106,7 +34690,7 @@
         <v>167.36</v>
       </c>
       <c r="G2368" t="n">
-        <v>54091.1</v>
+        <v>53907.48281973042</v>
       </c>
     </row>
     <row r="2369">
@@ -34120,7 +34704,7 @@
         <v>166.86</v>
       </c>
       <c r="G2369" t="n">
-        <v>57556.3</v>
+        <v>53522.12947632837</v>
       </c>
     </row>
     <row r="2370">
@@ -34134,7 +34718,7 @@
         <v>166.36</v>
       </c>
       <c r="G2370" t="n">
-        <v>57985.1</v>
+        <v>53137.36617520232</v>
       </c>
     </row>
     <row r="2371">
@@ -34148,7 +34732,7 @@
         <v>165.86</v>
       </c>
       <c r="G2371" t="n">
-        <v>58692.7</v>
+        <v>52754.20562342993</v>
       </c>
     </row>
     <row r="2372">
@@ -34162,7 +34746,7 @@
         <v>165.36</v>
       </c>
       <c r="G2372" t="n">
-        <v>56275.9</v>
+        <v>52373.92485887194</v>
       </c>
     </row>
     <row r="2373">
@@ -34176,7 +34760,7 @@
         <v>164.86</v>
       </c>
       <c r="G2373" t="n">
-        <v>59590.8</v>
+        <v>51994.97434763859</v>
       </c>
     </row>
     <row r="2374">
@@ -34190,7 +34774,7 @@
         <v>164.36</v>
       </c>
       <c r="G2374" t="n">
-        <v>63625.3</v>
+        <v>51621.0132265279</v>
       </c>
     </row>
     <row r="2375">
@@ -34204,7 +34788,7 @@
         <v>163.86</v>
       </c>
       <c r="G2375" t="n">
-        <v>71654.8</v>
+        <v>51256.35434033174</v>
       </c>
     </row>
     <row r="2376">
@@ -34218,7 +34802,7 @@
         <v>163.36</v>
       </c>
       <c r="G2376" t="n">
-        <v>84296.2</v>
+        <v>50908.92607005282</v>
       </c>
     </row>
     <row r="2377">
@@ -34232,7 +34816,7 @@
         <v>162.86</v>
       </c>
       <c r="G2377" t="n">
-        <v>101874</v>
+        <v>50590.81586409064</v>
       </c>
     </row>
     <row r="2378">
@@ -34246,7 +34830,7 @@
         <v>162.36</v>
       </c>
       <c r="G2378" t="n">
-        <v>119892</v>
+        <v>50318.54095397885</v>
       </c>
     </row>
     <row r="2379">
@@ -34260,7 +34844,7 @@
         <v>161.86</v>
       </c>
       <c r="G2379" t="n">
-        <v>127005</v>
+        <v>50108.93796497837</v>
       </c>
     </row>
     <row r="2380">
@@ -34274,7 +34858,7 @@
         <v>161.36</v>
       </c>
       <c r="G2380" t="n">
-        <v>121387</v>
+        <v>49968.83903380438</v>
       </c>
     </row>
     <row r="2381">
@@ -34288,7 +34872,7 @@
         <v>160.86</v>
       </c>
       <c r="G2381" t="n">
-        <v>95260</v>
+        <v>49893.4018597074</v>
       </c>
     </row>
     <row r="2382">
@@ -34302,7 +34886,7 @@
         <v>160.36</v>
       </c>
       <c r="G2382" t="n">
-        <v>74102.8</v>
+        <v>49859.06200159782</v>
       </c>
     </row>
     <row r="2383">
@@ -34316,7 +34900,7 @@
         <v>159.86</v>
       </c>
       <c r="G2383" t="n">
-        <v>57571.8</v>
+        <v>49846.68872254089</v>
       </c>
     </row>
     <row r="2384">
@@ -34330,7 +34914,7 @@
         <v>159.36</v>
       </c>
       <c r="G2384" t="n">
-        <v>51619.9</v>
+        <v>49841.30802674772</v>
       </c>
     </row>
     <row r="2385">
@@ -34344,7 +34928,7 @@
         <v>158.86</v>
       </c>
       <c r="G2385" t="n">
-        <v>51900.9</v>
+        <v>49837.53012317182</v>
       </c>
     </row>
     <row r="2386">
@@ -34358,7 +34942,7 @@
         <v>158.36</v>
       </c>
       <c r="G2386" t="n">
-        <v>51094.5</v>
+        <v>49835.61655719589</v>
       </c>
     </row>
     <row r="2387">
@@ -34372,7 +34956,7 @@
         <v>157.86</v>
       </c>
       <c r="G2387" t="n">
-        <v>51191.3</v>
+        <v>49834.83906969597</v>
       </c>
     </row>
     <row r="2388">
@@ -34386,7 +34970,7 @@
         <v>157.36</v>
       </c>
       <c r="G2388" t="n">
-        <v>50027.5</v>
+        <v>49835.28670095154</v>
       </c>
     </row>
     <row r="2389">
@@ -34400,7 +34984,7 @@
         <v>156.86</v>
       </c>
       <c r="G2389" t="n">
-        <v>48774.5</v>
+        <v>49835.90272391577</v>
       </c>
     </row>
     <row r="2390">
@@ -34414,7 +34998,7 @@
         <v>156.36</v>
       </c>
       <c r="G2390" t="n">
-        <v>47102.5</v>
+        <v>49835.54921726152</v>
       </c>
     </row>
     <row r="2391">
@@ -34428,7 +35012,7 @@
         <v>155.86</v>
       </c>
       <c r="G2391" t="n">
-        <v>52289.4</v>
+        <v>49832.7099659503</v>
       </c>
     </row>
     <row r="2392">
@@ -34442,7 +35026,7 @@
         <v>155.36</v>
       </c>
       <c r="G2392" t="n">
-        <v>49613.1</v>
+        <v>49832.09541036117</v>
       </c>
     </row>
     <row r="2393">
@@ -34456,7 +35040,7 @@
         <v>154.86</v>
       </c>
       <c r="G2393" t="n">
-        <v>49465.8</v>
+        <v>49831.27881146793</v>
       </c>
     </row>
     <row r="2394">
@@ -34470,7 +35054,7 @@
         <v>154.36</v>
       </c>
       <c r="G2394" t="n">
-        <v>50241.6</v>
+        <v>49830.12801232468</v>
       </c>
     </row>
     <row r="2395">
@@ -34484,7 +35068,7 @@
         <v>153.86</v>
       </c>
       <c r="G2395" t="n">
-        <v>49678.9</v>
+        <v>49829.34887500744</v>
       </c>
     </row>
     <row r="2396">
@@ -34498,7 +35082,7 @@
         <v>153.36</v>
       </c>
       <c r="G2396" t="n">
-        <v>50823.5</v>
+        <v>49828.43236529823</v>
       </c>
     </row>
     <row r="2397">
@@ -34512,7 +35096,7 @@
         <v>152.86</v>
       </c>
       <c r="G2397" t="n">
-        <v>49516.6</v>
+        <v>49828.4184903645</v>
       </c>
     </row>
     <row r="2398">
@@ -34526,7 +35110,7 @@
         <v>152.36</v>
       </c>
       <c r="G2398" t="n">
-        <v>49453.7</v>
+        <v>49828.12172028612</v>
       </c>
     </row>
     <row r="2399">
@@ -34540,7 +35124,7 @@
         <v>151.86</v>
       </c>
       <c r="G2399" t="n">
-        <v>51535.9</v>
+        <v>49827.48554234149</v>
       </c>
     </row>
     <row r="2400">
@@ -34554,7 +35138,7 @@
         <v>151.36</v>
       </c>
       <c r="G2400" t="n">
-        <v>47812.3</v>
+        <v>49828.4</v>
       </c>
     </row>
     <row r="2401">
@@ -39067,7 +39651,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="X2:AQ2"/>
+    <mergeCell ref="X10:AQ10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>